<commit_message>
At home holiday work
</commit_message>
<xml_diff>
--- a/Flowtracker_Nektar.xlsx
+++ b/Flowtracker_Nektar.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28025"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cbnor\Documents\Full Body Flow Model Project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C160F398-35A7-4B1D-A756-38A72A986ABA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1F902B5-99E8-448E-B6FD-A8D061EE7A51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{1D1F38B3-363E-4804-8520-607C8FB177D0}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{1D1F38B3-363E-4804-8520-607C8FB177D0}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -525,15 +525,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{70DF22C3-18CC-477F-9A54-36AC51B31683}">
   <dimension ref="A1:D28"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
-    <col min="2" max="2" width="18.28515625" customWidth="1"/>
-    <col min="3" max="3" width="36.28515625" customWidth="1"/>
-    <col min="4" max="4" width="18.140625" customWidth="1"/>
+    <col min="2" max="2" width="18.265625" customWidth="1"/>
+    <col min="3" max="3" width="36.265625" customWidth="1"/>
+    <col min="4" max="4" width="18.1328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -547,7 +547,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -561,7 +561,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -575,7 +575,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>10</v>
       </c>
@@ -586,7 +586,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>11</v>
       </c>
@@ -597,7 +597,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -605,7 +605,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -613,7 +613,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>13</v>
       </c>
@@ -621,7 +621,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>14</v>
       </c>
@@ -635,7 +635,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
         <v>16</v>
       </c>
@@ -646,7 +646,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
         <v>17</v>
       </c>
@@ -657,7 +657,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
         <v>18</v>
       </c>
@@ -665,7 +665,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
         <v>19</v>
       </c>
@@ -676,7 +676,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
         <v>20</v>
       </c>
@@ -684,7 +684,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
         <v>22</v>
       </c>
@@ -692,7 +692,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
         <v>23</v>
       </c>
@@ -700,7 +700,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
         <v>24</v>
       </c>
@@ -708,7 +708,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
         <v>34</v>
       </c>
@@ -716,7 +716,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A19" t="s">
         <v>25</v>
       </c>
@@ -724,7 +724,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A20" t="s">
         <v>26</v>
       </c>
@@ -735,7 +735,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A21" t="s">
         <v>28</v>
       </c>
@@ -746,7 +746,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A22" t="s">
         <v>27</v>
       </c>
@@ -757,7 +757,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
         <v>29</v>
       </c>
@@ -768,7 +768,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A24" t="s">
         <v>30</v>
       </c>
@@ -776,7 +776,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A25" t="s">
         <v>37</v>
       </c>
@@ -784,7 +784,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A26" t="s">
         <v>35</v>
       </c>
@@ -792,7 +792,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A27" t="s">
         <v>32</v>
       </c>
@@ -800,7 +800,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A28" t="s">
         <v>33</v>
       </c>

</xml_diff>